<commit_message>
Update reference file: Y4_B2526_General_&_Special_Surgery_1_A1_reference_data.xlsx
</commit_message>
<xml_diff>
--- a/reference_data/Y4_B2526_General_&_Special_Surgery_1_A1_reference_data.xlsx
+++ b/reference_data/Y4_B2526_General_&_Special_Surgery_1_A1_reference_data.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E426"/>
+  <dimension ref="A1:E427"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -514,7 +514,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -541,7 +541,7 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -649,7 +649,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -703,7 +703,7 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -730,7 +730,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -784,7 +784,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -811,7 +811,7 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -838,7 +838,7 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -865,7 +865,7 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -919,7 +919,7 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -946,7 +946,7 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1000,7 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1027,7 +1027,7 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1054,7 +1054,7 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1108,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1162,7 +1162,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1243,7 +1243,7 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1270,7 +1270,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1297,7 +1297,7 @@
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1324,7 +1324,7 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1405,7 @@
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1432,7 +1432,7 @@
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1459,7 +1459,7 @@
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1486,7 +1486,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1513,7 +1513,7 @@
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1540,7 +1540,7 @@
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1567,7 +1567,7 @@
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1594,7 +1594,7 @@
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1621,7 @@
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1648,7 +1648,7 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1675,7 +1675,7 @@
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1702,7 +1702,7 @@
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1729,7 +1729,7 @@
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1756,7 +1756,7 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1783,7 +1783,7 @@
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1810,7 +1810,7 @@
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1837,7 +1837,7 @@
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1891,7 +1891,7 @@
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1918,7 +1918,7 @@
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1945,7 +1945,7 @@
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1972,7 +1972,7 @@
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -1999,7 +1999,7 @@
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2026,7 +2026,7 @@
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2053,7 @@
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2080,7 +2080,7 @@
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2107,7 +2107,7 @@
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2134,7 +2134,7 @@
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2161,7 +2161,7 @@
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2188,7 +2188,7 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2215,7 +2215,7 @@
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2242,7 +2242,7 @@
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2269,7 +2269,7 @@
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2296,7 +2296,7 @@
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2323,7 +2323,7 @@
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2350,7 +2350,7 @@
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2377,7 +2377,7 @@
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2404,7 @@
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2431,7 +2431,7 @@
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2458,7 +2458,7 @@
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2485,7 +2485,7 @@
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2539,7 +2539,7 @@
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2566,7 +2566,7 @@
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2593,7 +2593,7 @@
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2620,7 +2620,7 @@
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2647,7 +2647,7 @@
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2674,7 +2674,7 @@
       </c>
       <c r="E82" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2701,7 +2701,7 @@
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2728,7 +2728,7 @@
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2755,7 +2755,7 @@
       </c>
       <c r="E85" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2782,7 +2782,7 @@
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2809,7 +2809,7 @@
       </c>
       <c r="E87" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2836,7 +2836,7 @@
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2863,7 +2863,7 @@
       </c>
       <c r="E89" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2917,7 +2917,7 @@
       </c>
       <c r="E91" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2944,7 @@
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2971,7 +2971,7 @@
       </c>
       <c r="E93" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -2998,7 +2998,7 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3025,7 +3025,7 @@
       </c>
       <c r="E95" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3052,7 +3052,7 @@
       </c>
       <c r="E96" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3079,7 +3079,7 @@
       </c>
       <c r="E97" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3106,7 +3106,7 @@
       </c>
       <c r="E98" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="E99" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3160,7 +3160,7 @@
       </c>
       <c r="E100" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3187,7 +3187,7 @@
       </c>
       <c r="E101" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3214,7 +3214,7 @@
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3241,7 +3241,7 @@
       </c>
       <c r="E103" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3268,7 +3268,7 @@
       </c>
       <c r="E104" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3295,7 +3295,7 @@
       </c>
       <c r="E105" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3322,7 +3322,7 @@
       </c>
       <c r="E106" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3349,7 +3349,7 @@
       </c>
       <c r="E107" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3376,7 +3376,7 @@
       </c>
       <c r="E108" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3403,7 +3403,7 @@
       </c>
       <c r="E109" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3430,7 +3430,7 @@
       </c>
       <c r="E110" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3457,7 +3457,7 @@
       </c>
       <c r="E111" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3484,7 +3484,7 @@
       </c>
       <c r="E112" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3511,7 +3511,7 @@
       </c>
       <c r="E113" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3538,7 +3538,7 @@
       </c>
       <c r="E114" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3565,7 +3565,7 @@
       </c>
       <c r="E115" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3592,7 +3592,7 @@
       </c>
       <c r="E116" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3619,7 +3619,7 @@
       </c>
       <c r="E117" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3646,7 +3646,7 @@
       </c>
       <c r="E118" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3673,7 +3673,7 @@
       </c>
       <c r="E119" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3700,7 +3700,7 @@
       </c>
       <c r="E120" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3727,7 +3727,7 @@
       </c>
       <c r="E121" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3754,7 +3754,7 @@
       </c>
       <c r="E122" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3781,7 +3781,7 @@
       </c>
       <c r="E123" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="E124" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3835,7 +3835,7 @@
       </c>
       <c r="E125" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3862,7 +3862,7 @@
       </c>
       <c r="E126" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3889,7 +3889,7 @@
       </c>
       <c r="E127" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3916,7 +3916,7 @@
       </c>
       <c r="E128" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3943,7 +3943,7 @@
       </c>
       <c r="E129" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3970,7 +3970,7 @@
       </c>
       <c r="E130" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -3997,7 +3997,7 @@
       </c>
       <c r="E131" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4024,7 +4024,7 @@
       </c>
       <c r="E132" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4051,7 +4051,7 @@
       </c>
       <c r="E133" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4078,7 +4078,7 @@
       </c>
       <c r="E134" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4105,7 +4105,7 @@
       </c>
       <c r="E135" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4132,7 +4132,7 @@
       </c>
       <c r="E136" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4159,7 +4159,7 @@
       </c>
       <c r="E137" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4186,7 +4186,7 @@
       </c>
       <c r="E138" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4213,7 +4213,7 @@
       </c>
       <c r="E139" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4240,7 +4240,7 @@
       </c>
       <c r="E140" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4267,7 +4267,7 @@
       </c>
       <c r="E141" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4294,7 +4294,7 @@
       </c>
       <c r="E142" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4321,7 +4321,7 @@
       </c>
       <c r="E143" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4348,7 +4348,7 @@
       </c>
       <c r="E144" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4375,7 +4375,7 @@
       </c>
       <c r="E145" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4402,7 +4402,7 @@
       </c>
       <c r="E146" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4429,7 +4429,7 @@
       </c>
       <c r="E147" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4456,7 +4456,7 @@
       </c>
       <c r="E148" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4483,7 +4483,7 @@
       </c>
       <c r="E149" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4510,7 +4510,7 @@
       </c>
       <c r="E150" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4537,7 @@
       </c>
       <c r="E151" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4564,7 +4564,7 @@
       </c>
       <c r="E152" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4591,7 +4591,7 @@
       </c>
       <c r="E153" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4618,7 +4618,7 @@
       </c>
       <c r="E154" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4645,7 +4645,7 @@
       </c>
       <c r="E155" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4672,7 +4672,7 @@
       </c>
       <c r="E156" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4699,7 +4699,7 @@
       </c>
       <c r="E157" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4726,7 +4726,7 @@
       </c>
       <c r="E158" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4753,7 +4753,7 @@
       </c>
       <c r="E159" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4780,7 +4780,7 @@
       </c>
       <c r="E160" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4807,7 +4807,7 @@
       </c>
       <c r="E161" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4834,7 +4834,7 @@
       </c>
       <c r="E162" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4861,7 +4861,7 @@
       </c>
       <c r="E163" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4888,7 +4888,7 @@
       </c>
       <c r="E164" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4915,7 +4915,7 @@
       </c>
       <c r="E165" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4942,7 +4942,7 @@
       </c>
       <c r="E166" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4969,7 +4969,7 @@
       </c>
       <c r="E167" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -4996,7 +4996,7 @@
       </c>
       <c r="E168" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5023,7 +5023,7 @@
       </c>
       <c r="E169" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5050,7 +5050,7 @@
       </c>
       <c r="E170" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5077,7 +5077,7 @@
       </c>
       <c r="E171" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5104,7 +5104,7 @@
       </c>
       <c r="E172" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5131,7 +5131,7 @@
       </c>
       <c r="E173" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5158,7 +5158,7 @@
       </c>
       <c r="E174" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5185,7 +5185,7 @@
       </c>
       <c r="E175" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5212,7 +5212,7 @@
       </c>
       <c r="E176" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5239,7 +5239,7 @@
       </c>
       <c r="E177" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5266,7 +5266,7 @@
       </c>
       <c r="E178" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5293,7 +5293,7 @@
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5320,7 +5320,7 @@
       </c>
       <c r="E180" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5347,7 +5347,7 @@
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5374,7 +5374,7 @@
       </c>
       <c r="E182" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5401,7 +5401,7 @@
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5428,7 +5428,7 @@
       </c>
       <c r="E184" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5455,7 +5455,7 @@
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5482,7 +5482,7 @@
       </c>
       <c r="E186" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5509,7 +5509,7 @@
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5536,7 +5536,7 @@
       </c>
       <c r="E188" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5563,7 +5563,7 @@
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5590,7 +5590,7 @@
       </c>
       <c r="E190" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5617,7 +5617,7 @@
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5644,7 +5644,7 @@
       </c>
       <c r="E192" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5671,7 +5671,7 @@
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5698,7 +5698,7 @@
       </c>
       <c r="E194" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5725,7 +5725,7 @@
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5752,7 +5752,7 @@
       </c>
       <c r="E196" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5779,7 +5779,7 @@
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5806,7 +5806,7 @@
       </c>
       <c r="E198" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5833,7 +5833,7 @@
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5860,7 +5860,7 @@
       </c>
       <c r="E200" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5887,7 +5887,7 @@
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5914,7 +5914,7 @@
       </c>
       <c r="E202" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5941,7 +5941,7 @@
       </c>
       <c r="E203" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5968,7 +5968,7 @@
       </c>
       <c r="E204" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -5995,7 +5995,7 @@
       </c>
       <c r="E205" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6022,7 +6022,7 @@
       </c>
       <c r="E206" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6049,7 +6049,7 @@
       </c>
       <c r="E207" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6076,7 +6076,7 @@
       </c>
       <c r="E208" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6103,7 +6103,7 @@
       </c>
       <c r="E209" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6130,7 +6130,7 @@
       </c>
       <c r="E210" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6157,7 +6157,7 @@
       </c>
       <c r="E211" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6184,7 +6184,7 @@
       </c>
       <c r="E212" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6211,7 +6211,7 @@
       </c>
       <c r="E213" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6238,7 +6238,7 @@
       </c>
       <c r="E214" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6265,7 +6265,7 @@
       </c>
       <c r="E215" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6292,7 +6292,7 @@
       </c>
       <c r="E216" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6319,7 +6319,7 @@
       </c>
       <c r="E217" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6346,7 +6346,7 @@
       </c>
       <c r="E218" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6373,7 +6373,7 @@
       </c>
       <c r="E219" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6400,7 +6400,7 @@
       </c>
       <c r="E220" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6427,7 +6427,7 @@
       </c>
       <c r="E221" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6454,7 +6454,7 @@
       </c>
       <c r="E222" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6481,7 +6481,7 @@
       </c>
       <c r="E223" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6508,7 +6508,7 @@
       </c>
       <c r="E224" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6535,7 +6535,7 @@
       </c>
       <c r="E225" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6562,7 +6562,7 @@
       </c>
       <c r="E226" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6589,7 +6589,7 @@
       </c>
       <c r="E227" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6616,7 +6616,7 @@
       </c>
       <c r="E228" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6643,7 +6643,7 @@
       </c>
       <c r="E229" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6670,7 +6670,7 @@
       </c>
       <c r="E230" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6697,7 +6697,7 @@
       </c>
       <c r="E231" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6724,7 +6724,7 @@
       </c>
       <c r="E232" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6751,7 +6751,7 @@
       </c>
       <c r="E233" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6778,7 +6778,7 @@
       </c>
       <c r="E234" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6805,7 +6805,7 @@
       </c>
       <c r="E235" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6832,7 +6832,7 @@
       </c>
       <c r="E236" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6859,7 +6859,7 @@
       </c>
       <c r="E237" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6886,7 +6886,7 @@
       </c>
       <c r="E238" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6913,7 +6913,7 @@
       </c>
       <c r="E239" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6940,7 +6940,7 @@
       </c>
       <c r="E240" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6967,7 +6967,7 @@
       </c>
       <c r="E241" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -6994,7 +6994,7 @@
       </c>
       <c r="E242" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7021,7 +7021,7 @@
       </c>
       <c r="E243" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7048,7 +7048,7 @@
       </c>
       <c r="E244" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7075,7 +7075,7 @@
       </c>
       <c r="E245" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7102,7 +7102,7 @@
       </c>
       <c r="E246" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7129,7 +7129,7 @@
       </c>
       <c r="E247" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7156,7 +7156,7 @@
       </c>
       <c r="E248" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7183,7 +7183,7 @@
       </c>
       <c r="E249" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7210,7 +7210,7 @@
       </c>
       <c r="E250" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7237,7 +7237,7 @@
       </c>
       <c r="E251" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7264,7 +7264,7 @@
       </c>
       <c r="E252" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7291,7 +7291,7 @@
       </c>
       <c r="E253" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7318,7 +7318,7 @@
       </c>
       <c r="E254" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7345,7 +7345,7 @@
       </c>
       <c r="E255" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7372,7 +7372,7 @@
       </c>
       <c r="E256" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7399,7 +7399,7 @@
       </c>
       <c r="E257" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7426,7 +7426,7 @@
       </c>
       <c r="E258" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7453,7 +7453,7 @@
       </c>
       <c r="E259" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7480,7 +7480,7 @@
       </c>
       <c r="E260" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7507,7 +7507,7 @@
       </c>
       <c r="E261" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7534,7 +7534,7 @@
       </c>
       <c r="E262" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7561,7 +7561,7 @@
       </c>
       <c r="E263" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7588,7 +7588,7 @@
       </c>
       <c r="E264" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7615,7 +7615,7 @@
       </c>
       <c r="E265" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7642,7 +7642,7 @@
       </c>
       <c r="E266" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7669,7 +7669,7 @@
       </c>
       <c r="E267" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7696,7 +7696,7 @@
       </c>
       <c r="E268" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7723,7 +7723,7 @@
       </c>
       <c r="E269" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7750,7 +7750,7 @@
       </c>
       <c r="E270" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7777,7 +7777,7 @@
       </c>
       <c r="E271" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7804,7 +7804,7 @@
       </c>
       <c r="E272" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7831,7 +7831,7 @@
       </c>
       <c r="E273" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7858,7 +7858,7 @@
       </c>
       <c r="E274" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7885,7 +7885,7 @@
       </c>
       <c r="E275" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7912,7 +7912,7 @@
       </c>
       <c r="E276" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7939,7 +7939,7 @@
       </c>
       <c r="E277" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7966,7 +7966,7 @@
       </c>
       <c r="E278" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -7993,7 +7993,7 @@
       </c>
       <c r="E279" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8020,7 +8020,7 @@
       </c>
       <c r="E280" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8047,7 +8047,7 @@
       </c>
       <c r="E281" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8074,7 +8074,7 @@
       </c>
       <c r="E282" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8101,7 +8101,7 @@
       </c>
       <c r="E283" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8128,7 +8128,7 @@
       </c>
       <c r="E284" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8155,7 +8155,7 @@
       </c>
       <c r="E285" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8182,7 +8182,7 @@
       </c>
       <c r="E286" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8209,7 +8209,7 @@
       </c>
       <c r="E287" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8236,7 +8236,7 @@
       </c>
       <c r="E288" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8263,7 +8263,7 @@
       </c>
       <c r="E289" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8290,7 +8290,7 @@
       </c>
       <c r="E290" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8317,7 +8317,7 @@
       </c>
       <c r="E291" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8344,7 +8344,7 @@
       </c>
       <c r="E292" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8371,7 +8371,7 @@
       </c>
       <c r="E293" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8398,7 +8398,7 @@
       </c>
       <c r="E294" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8425,7 +8425,7 @@
       </c>
       <c r="E295" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8452,7 +8452,7 @@
       </c>
       <c r="E296" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8479,7 +8479,7 @@
       </c>
       <c r="E297" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8506,7 +8506,7 @@
       </c>
       <c r="E298" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8533,7 +8533,7 @@
       </c>
       <c r="E299" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8560,7 +8560,7 @@
       </c>
       <c r="E300" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8587,7 +8587,7 @@
       </c>
       <c r="E301" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8614,7 +8614,7 @@
       </c>
       <c r="E302" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8641,7 +8641,7 @@
       </c>
       <c r="E303" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8668,7 +8668,7 @@
       </c>
       <c r="E304" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8695,7 +8695,7 @@
       </c>
       <c r="E305" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8722,7 +8722,7 @@
       </c>
       <c r="E306" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8749,7 +8749,7 @@
       </c>
       <c r="E307" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8776,7 +8776,7 @@
       </c>
       <c r="E308" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8803,7 +8803,7 @@
       </c>
       <c r="E309" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8830,7 +8830,7 @@
       </c>
       <c r="E310" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8857,7 +8857,7 @@
       </c>
       <c r="E311" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8884,7 +8884,7 @@
       </c>
       <c r="E312" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8911,7 +8911,7 @@
       </c>
       <c r="E313" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8938,7 +8938,7 @@
       </c>
       <c r="E314" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8965,7 +8965,7 @@
       </c>
       <c r="E315" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -8992,7 +8992,7 @@
       </c>
       <c r="E316" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9019,7 +9019,7 @@
       </c>
       <c r="E317" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9046,7 +9046,7 @@
       </c>
       <c r="E318" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9073,7 +9073,7 @@
       </c>
       <c r="E319" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9100,7 +9100,7 @@
       </c>
       <c r="E320" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9127,7 +9127,7 @@
       </c>
       <c r="E321" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9154,7 +9154,7 @@
       </c>
       <c r="E322" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9181,7 +9181,7 @@
       </c>
       <c r="E323" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9208,7 +9208,7 @@
       </c>
       <c r="E324" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9235,7 +9235,7 @@
       </c>
       <c r="E325" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9262,7 +9262,7 @@
       </c>
       <c r="E326" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9289,7 +9289,7 @@
       </c>
       <c r="E327" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9316,7 +9316,7 @@
       </c>
       <c r="E328" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9343,7 +9343,7 @@
       </c>
       <c r="E329" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9370,7 +9370,7 @@
       </c>
       <c r="E330" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9397,7 +9397,7 @@
       </c>
       <c r="E331" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9424,7 +9424,7 @@
       </c>
       <c r="E332" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9451,7 +9451,7 @@
       </c>
       <c r="E333" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9478,7 +9478,7 @@
       </c>
       <c r="E334" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9505,7 +9505,7 @@
       </c>
       <c r="E335" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9532,7 +9532,7 @@
       </c>
       <c r="E336" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9559,7 +9559,7 @@
       </c>
       <c r="E337" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9586,7 +9586,7 @@
       </c>
       <c r="E338" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9613,7 +9613,7 @@
       </c>
       <c r="E339" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9640,7 +9640,7 @@
       </c>
       <c r="E340" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9667,7 +9667,7 @@
       </c>
       <c r="E341" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9694,7 +9694,7 @@
       </c>
       <c r="E342" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9721,7 +9721,7 @@
       </c>
       <c r="E343" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9748,7 +9748,7 @@
       </c>
       <c r="E344" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9775,7 +9775,7 @@
       </c>
       <c r="E345" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9802,7 +9802,7 @@
       </c>
       <c r="E346" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9829,7 +9829,7 @@
       </c>
       <c r="E347" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9856,7 +9856,7 @@
       </c>
       <c r="E348" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9883,7 +9883,7 @@
       </c>
       <c r="E349" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9910,7 +9910,7 @@
       </c>
       <c r="E350" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9937,7 +9937,7 @@
       </c>
       <c r="E351" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9964,7 +9964,7 @@
       </c>
       <c r="E352" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -9991,7 +9991,7 @@
       </c>
       <c r="E353" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -10018,7 +10018,7 @@
       </c>
       <c r="E354" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -10045,7 +10045,7 @@
       </c>
       <c r="E355" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -10072,7 +10072,7 @@
       </c>
       <c r="E356" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -10099,7 +10099,7 @@
       </c>
       <c r="E357" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -10126,7 +10126,7 @@
       </c>
       <c r="E358" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -10153,7 +10153,7 @@
       </c>
       <c r="E359" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -10180,7 +10180,7 @@
       </c>
       <c r="E360" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
@@ -10207,19 +10207,19 @@
       </c>
       <c r="E361" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" s="3" t="inlineStr">
         <is>
-          <t>211993</t>
+          <t>211966</t>
         </is>
       </c>
       <c r="B362" s="3" t="inlineStr">
         <is>
-          <t>Sidra Parvez</t>
+          <t>Malony Ngong Deng Maathiei</t>
         </is>
       </c>
       <c r="C362" s="3" t="inlineStr">
@@ -10234,19 +10234,19 @@
       </c>
       <c r="E362" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" s="4" t="inlineStr">
         <is>
-          <t>212148</t>
+          <t>211993</t>
         </is>
       </c>
       <c r="B363" s="4" t="inlineStr">
         <is>
-          <t>عائشه بيبى فاروق</t>
+          <t>Sidra Parvez</t>
         </is>
       </c>
       <c r="C363" s="4" t="inlineStr">
@@ -10261,19 +10261,19 @@
       </c>
       <c r="E363" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" s="3" t="inlineStr">
         <is>
-          <t>212181</t>
+          <t>212148</t>
         </is>
       </c>
       <c r="B364" s="3" t="inlineStr">
         <is>
-          <t>موسكان لطيف</t>
+          <t>عائشه بيبى فاروق</t>
         </is>
       </c>
       <c r="C364" s="3" t="inlineStr">
@@ -10288,19 +10288,19 @@
       </c>
       <c r="E364" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" s="4" t="inlineStr">
         <is>
-          <t>212197</t>
+          <t>212181</t>
         </is>
       </c>
       <c r="B365" s="4" t="inlineStr">
         <is>
-          <t>Syeda Hafsa Batool</t>
+          <t>موسكان لطيف</t>
         </is>
       </c>
       <c r="C365" s="4" t="inlineStr">
@@ -10315,19 +10315,19 @@
       </c>
       <c r="E365" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" s="3" t="inlineStr">
         <is>
-          <t>212223</t>
+          <t>212197</t>
         </is>
       </c>
       <c r="B366" s="3" t="inlineStr">
         <is>
-          <t>Dhanush Kumar Udhayakumar</t>
+          <t>Syeda Hafsa Batool</t>
         </is>
       </c>
       <c r="C366" s="3" t="inlineStr">
@@ -10342,19 +10342,19 @@
       </c>
       <c r="E366" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" s="4" t="inlineStr">
         <is>
-          <t>212230</t>
+          <t>212223</t>
         </is>
       </c>
       <c r="B367" s="4" t="inlineStr">
         <is>
-          <t>Mohammed Mufeed</t>
+          <t>Dhanush Kumar Udhayakumar</t>
         </is>
       </c>
       <c r="C367" s="4" t="inlineStr">
@@ -10369,19 +10369,19 @@
       </c>
       <c r="E367" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" s="3" t="inlineStr">
         <is>
-          <t>212234</t>
+          <t>212230</t>
         </is>
       </c>
       <c r="B368" s="3" t="inlineStr">
         <is>
-          <t>Mirrah Naseer</t>
+          <t>Mohammed Mufeed</t>
         </is>
       </c>
       <c r="C368" s="3" t="inlineStr">
@@ -10396,19 +10396,19 @@
       </c>
       <c r="E368" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" s="4" t="inlineStr">
         <is>
-          <t>212239</t>
+          <t>212234</t>
         </is>
       </c>
       <c r="B369" s="4" t="inlineStr">
         <is>
-          <t>حليمه تاسع</t>
+          <t>Mirrah Naseer</t>
         </is>
       </c>
       <c r="C369" s="4" t="inlineStr">
@@ -10423,19 +10423,19 @@
       </c>
       <c r="E369" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" s="3" t="inlineStr">
         <is>
-          <t>212281</t>
+          <t>212239</t>
         </is>
       </c>
       <c r="B370" s="3" t="inlineStr">
         <is>
-          <t>Athiei Chol Chan Chol</t>
+          <t>حليمه تاسع</t>
         </is>
       </c>
       <c r="C370" s="3" t="inlineStr">
@@ -10450,19 +10450,19 @@
       </c>
       <c r="E370" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" s="4" t="inlineStr">
         <is>
-          <t>212437</t>
+          <t>212281</t>
         </is>
       </c>
       <c r="B371" s="4" t="inlineStr">
         <is>
-          <t>حبيبة بيلجور</t>
+          <t>Athiei Chol Chan Chol</t>
         </is>
       </c>
       <c r="C371" s="4" t="inlineStr">
@@ -10477,19 +10477,19 @@
       </c>
       <c r="E371" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" s="3" t="inlineStr">
         <is>
-          <t>212574</t>
+          <t>212437</t>
         </is>
       </c>
       <c r="B372" s="3" t="inlineStr">
         <is>
-          <t>اديمولا محمد مصطفى</t>
+          <t>حبيبة بيلجور</t>
         </is>
       </c>
       <c r="C372" s="3" t="inlineStr">
@@ -10504,19 +10504,19 @@
       </c>
       <c r="E372" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" s="4" t="inlineStr">
         <is>
-          <t>220551</t>
+          <t>212574</t>
         </is>
       </c>
       <c r="B373" s="4" t="inlineStr">
         <is>
-          <t>صاليف سيريس</t>
+          <t>اديمولا محمد مصطفى</t>
         </is>
       </c>
       <c r="C373" s="4" t="inlineStr">
@@ -10531,19 +10531,19 @@
       </c>
       <c r="E373" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="374">
       <c r="A374" s="3" t="inlineStr">
         <is>
-          <t>220565</t>
+          <t>220551</t>
         </is>
       </c>
       <c r="B374" s="3" t="inlineStr">
         <is>
-          <t>عبد القادر خزيمه بيثهاوالا</t>
+          <t>صاليف سيريس</t>
         </is>
       </c>
       <c r="C374" s="3" t="inlineStr">
@@ -10558,19 +10558,19 @@
       </c>
       <c r="E374" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="375">
       <c r="A375" s="4" t="inlineStr">
         <is>
-          <t>220886</t>
+          <t>220565</t>
         </is>
       </c>
       <c r="B375" s="4" t="inlineStr">
         <is>
-          <t>عائشه حافظ مجيب الرحمان حافظ جمشيد علي فرقان</t>
+          <t>عبد القادر خزيمه بيثهاوالا</t>
         </is>
       </c>
       <c r="C375" s="4" t="inlineStr">
@@ -10585,19 +10585,19 @@
       </c>
       <c r="E375" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="376">
       <c r="A376" s="3" t="inlineStr">
         <is>
-          <t>220887</t>
+          <t>220886</t>
         </is>
       </c>
       <c r="B376" s="3" t="inlineStr">
         <is>
-          <t>رافة خنساء احمد عبد الله محمد روية</t>
+          <t>عائشه حافظ مجيب الرحمان حافظ جمشيد علي فرقان</t>
         </is>
       </c>
       <c r="C376" s="3" t="inlineStr">
@@ -10612,19 +10612,19 @@
       </c>
       <c r="E376" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="377">
       <c r="A377" s="4" t="inlineStr">
         <is>
-          <t>221003</t>
+          <t>220887</t>
         </is>
       </c>
       <c r="B377" s="4" t="inlineStr">
         <is>
-          <t>مريم عبدالرحمن يحيى</t>
+          <t>رافة خنساء احمد عبد الله محمد روية</t>
         </is>
       </c>
       <c r="C377" s="4" t="inlineStr">
@@ -10639,19 +10639,19 @@
       </c>
       <c r="E377" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" s="3" t="inlineStr">
         <is>
-          <t>221042</t>
+          <t>221003</t>
         </is>
       </c>
       <c r="B378" s="3" t="inlineStr">
         <is>
-          <t>ادم حسينى بوهرا</t>
+          <t>مريم عبدالرحمن يحيى</t>
         </is>
       </c>
       <c r="C378" s="3" t="inlineStr">
@@ -10666,19 +10666,19 @@
       </c>
       <c r="E378" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" s="4" t="inlineStr">
         <is>
-          <t>221446</t>
+          <t>221042</t>
         </is>
       </c>
       <c r="B379" s="4" t="inlineStr">
         <is>
-          <t>بلقس يحي نجم</t>
+          <t>ادم حسينى بوهرا</t>
         </is>
       </c>
       <c r="C379" s="4" t="inlineStr">
@@ -10693,19 +10693,19 @@
       </c>
       <c r="E379" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" s="3" t="inlineStr">
         <is>
-          <t>221449</t>
+          <t>221446</t>
         </is>
       </c>
       <c r="B380" s="3" t="inlineStr">
         <is>
-          <t>سهلة فاطمة بدر</t>
+          <t>بلقس يحي نجم</t>
         </is>
       </c>
       <c r="C380" s="3" t="inlineStr">
@@ -10720,19 +10720,19 @@
       </c>
       <c r="E380" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" s="4" t="inlineStr">
         <is>
-          <t>221513</t>
+          <t>221449</t>
         </is>
       </c>
       <c r="B381" s="4" t="inlineStr">
         <is>
-          <t>جميلة قائد جوهر جادي والا</t>
+          <t>سهلة فاطمة بدر</t>
         </is>
       </c>
       <c r="C381" s="4" t="inlineStr">
@@ -10747,19 +10747,19 @@
       </c>
       <c r="E381" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" s="3" t="inlineStr">
         <is>
-          <t>221723</t>
+          <t>221513</t>
         </is>
       </c>
       <c r="B382" s="3" t="inlineStr">
         <is>
-          <t>Nahla Sherin Moolayil</t>
+          <t>جميلة قائد جوهر جادي والا</t>
         </is>
       </c>
       <c r="C382" s="3" t="inlineStr">
@@ -10774,19 +10774,19 @@
       </c>
       <c r="E382" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" s="4" t="inlineStr">
         <is>
-          <t>222041</t>
+          <t>221723</t>
         </is>
       </c>
       <c r="B383" s="4" t="inlineStr">
         <is>
-          <t>Shahala Suhara Manzil</t>
+          <t>Nahla Sherin Moolayil</t>
         </is>
       </c>
       <c r="C383" s="4" t="inlineStr">
@@ -10801,19 +10801,19 @@
       </c>
       <c r="E383" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="A384" s="3" t="inlineStr">
         <is>
-          <t>222054</t>
+          <t>222041</t>
         </is>
       </c>
       <c r="B384" s="3" t="inlineStr">
         <is>
-          <t>صديق ابراهيم</t>
+          <t>Shahala Suhara Manzil</t>
         </is>
       </c>
       <c r="C384" s="3" t="inlineStr">
@@ -10828,19 +10828,19 @@
       </c>
       <c r="E384" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="A385" s="4" t="inlineStr">
         <is>
-          <t>222073</t>
+          <t>222054</t>
         </is>
       </c>
       <c r="B385" s="4" t="inlineStr">
         <is>
-          <t>Aisha Aremu Olasubomi</t>
+          <t>صديق ابراهيم</t>
         </is>
       </c>
       <c r="C385" s="4" t="inlineStr">
@@ -10855,19 +10855,19 @@
       </c>
       <c r="E385" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="A386" s="3" t="inlineStr">
         <is>
-          <t>222117</t>
+          <t>222073</t>
         </is>
       </c>
       <c r="B386" s="3" t="inlineStr">
         <is>
-          <t>راهول لالان شوراسيا</t>
+          <t>Aisha Aremu Olasubomi</t>
         </is>
       </c>
       <c r="C386" s="3" t="inlineStr">
@@ -10882,19 +10882,19 @@
       </c>
       <c r="E386" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" s="4" t="inlineStr">
         <is>
-          <t>222122</t>
+          <t>222117</t>
         </is>
       </c>
       <c r="B387" s="4" t="inlineStr">
         <is>
-          <t>Madhumitha Rathinasamy</t>
+          <t>راهول لالان شوراسيا</t>
         </is>
       </c>
       <c r="C387" s="4" t="inlineStr">
@@ -10909,19 +10909,19 @@
       </c>
       <c r="E387" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" s="3" t="inlineStr">
         <is>
-          <t>200994</t>
+          <t>222122</t>
         </is>
       </c>
       <c r="B388" s="3" t="inlineStr">
         <is>
-          <t>مريم عبد الرزاق جامع</t>
+          <t>Madhumitha Rathinasamy</t>
         </is>
       </c>
       <c r="C388" s="3" t="inlineStr">
@@ -10931,24 +10931,24 @@
       </c>
       <c r="D388" s="3" t="inlineStr">
         <is>
-          <t>A1-F2</t>
+          <t>A1-F1</t>
         </is>
       </c>
       <c r="E388" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" s="4" t="inlineStr">
         <is>
-          <t>201227</t>
+          <t>200994</t>
         </is>
       </c>
       <c r="B389" s="4" t="inlineStr">
         <is>
-          <t>اميد داك سلمون</t>
+          <t>مريم عبد الرزاق جامع</t>
         </is>
       </c>
       <c r="C389" s="4" t="inlineStr">
@@ -10963,19 +10963,19 @@
       </c>
       <c r="E389" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" s="3" t="inlineStr">
         <is>
-          <t>201427</t>
+          <t>201227</t>
         </is>
       </c>
       <c r="B390" s="3" t="inlineStr">
         <is>
-          <t>رانو مهتا</t>
+          <t>اميد داك سلمون</t>
         </is>
       </c>
       <c r="C390" s="3" t="inlineStr">
@@ -10990,19 +10990,19 @@
       </c>
       <c r="E390" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" s="4" t="inlineStr">
         <is>
-          <t>201457</t>
+          <t>201427</t>
         </is>
       </c>
       <c r="B391" s="4" t="inlineStr">
         <is>
-          <t>عمار عظيم الدين سيد</t>
+          <t>رانو مهتا</t>
         </is>
       </c>
       <c r="C391" s="4" t="inlineStr">
@@ -11017,19 +11017,19 @@
       </c>
       <c r="E391" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" s="3" t="inlineStr">
         <is>
-          <t>201484</t>
+          <t>201457</t>
         </is>
       </c>
       <c r="B392" s="3" t="inlineStr">
         <is>
-          <t>لينا عامر احمد ابراهيم</t>
+          <t>عمار عظيم الدين سيد</t>
         </is>
       </c>
       <c r="C392" s="3" t="inlineStr">
@@ -11044,19 +11044,19 @@
       </c>
       <c r="E392" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" s="4" t="inlineStr">
         <is>
-          <t>201551</t>
+          <t>201484</t>
         </is>
       </c>
       <c r="B393" s="4" t="inlineStr">
         <is>
-          <t>Omkar Purushottam Karjule</t>
+          <t>لينا عامر احمد ابراهيم</t>
         </is>
       </c>
       <c r="C393" s="4" t="inlineStr">
@@ -11071,19 +11071,19 @@
       </c>
       <c r="E393" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" s="3" t="inlineStr">
         <is>
-          <t>201556</t>
+          <t>201551</t>
         </is>
       </c>
       <c r="B394" s="3" t="inlineStr">
         <is>
-          <t>عبد الرحمن اس ( عبد الرحمن شاك مجبور )</t>
+          <t>Omkar Purushottam Karjule</t>
         </is>
       </c>
       <c r="C394" s="3" t="inlineStr">
@@ -11098,19 +11098,19 @@
       </c>
       <c r="E394" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" s="4" t="inlineStr">
         <is>
-          <t>201804</t>
+          <t>201556</t>
         </is>
       </c>
       <c r="B395" s="4" t="inlineStr">
         <is>
-          <t>Vishnu Suraajhan Krishnan Rani</t>
+          <t>عبد الرحمن اس ( عبد الرحمن شاك مجبور )</t>
         </is>
       </c>
       <c r="C395" s="4" t="inlineStr">
@@ -11125,19 +11125,19 @@
       </c>
       <c r="E395" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" s="3" t="inlineStr">
         <is>
-          <t>201860</t>
+          <t>201804</t>
         </is>
       </c>
       <c r="B396" s="3" t="inlineStr">
         <is>
-          <t>فى وش نافى سرى</t>
+          <t>Vishnu Suraajhan Krishnan Rani</t>
         </is>
       </c>
       <c r="C396" s="3" t="inlineStr">
@@ -11152,19 +11152,19 @@
       </c>
       <c r="E396" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" s="4" t="inlineStr">
         <is>
-          <t>211972</t>
+          <t>201860</t>
         </is>
       </c>
       <c r="B397" s="4" t="inlineStr">
         <is>
-          <t>جاتلك سارجيس ويل</t>
+          <t>فى وش نافى سرى</t>
         </is>
       </c>
       <c r="C397" s="4" t="inlineStr">
@@ -11179,19 +11179,19 @@
       </c>
       <c r="E397" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" s="3" t="inlineStr">
         <is>
-          <t>211990</t>
+          <t>211972</t>
         </is>
       </c>
       <c r="B398" s="3" t="inlineStr">
         <is>
-          <t>Ageth Charles Chan Awang</t>
+          <t>جاتلك سارجيس ويل</t>
         </is>
       </c>
       <c r="C398" s="3" t="inlineStr">
@@ -11206,19 +11206,19 @@
       </c>
       <c r="E398" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" s="4" t="inlineStr">
         <is>
-          <t>212097</t>
+          <t>211990</t>
         </is>
       </c>
       <c r="B399" s="4" t="inlineStr">
         <is>
-          <t>Preeti</t>
+          <t>Ageth Charles Chan Awang</t>
         </is>
       </c>
       <c r="C399" s="4" t="inlineStr">
@@ -11233,19 +11233,19 @@
       </c>
       <c r="E399" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" s="3" t="inlineStr">
         <is>
-          <t>212103</t>
+          <t>212097</t>
         </is>
       </c>
       <c r="B400" s="3" t="inlineStr">
         <is>
-          <t>Azim Ahmed Basheer Athira</t>
+          <t>Preeti</t>
         </is>
       </c>
       <c r="C400" s="3" t="inlineStr">
@@ -11260,19 +11260,19 @@
       </c>
       <c r="E400" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" s="4" t="inlineStr">
         <is>
-          <t>212114</t>
+          <t>212103</t>
         </is>
       </c>
       <c r="B401" s="4" t="inlineStr">
         <is>
-          <t>Samar Jan</t>
+          <t>Azim Ahmed Basheer Athira</t>
         </is>
       </c>
       <c r="C401" s="4" t="inlineStr">
@@ -11287,19 +11287,19 @@
       </c>
       <c r="E401" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" s="3" t="inlineStr">
         <is>
-          <t>212116</t>
+          <t>212114</t>
         </is>
       </c>
       <c r="B402" s="3" t="inlineStr">
         <is>
-          <t>Madbean Charles Chan Awang</t>
+          <t>Samar Jan</t>
         </is>
       </c>
       <c r="C402" s="3" t="inlineStr">
@@ -11314,19 +11314,19 @@
       </c>
       <c r="E402" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" s="4" t="inlineStr">
         <is>
-          <t>212133</t>
+          <t>212116</t>
         </is>
       </c>
       <c r="B403" s="4" t="inlineStr">
         <is>
-          <t>Mohammed Kashif Saleem</t>
+          <t>Madbean Charles Chan Awang</t>
         </is>
       </c>
       <c r="C403" s="4" t="inlineStr">
@@ -11341,19 +11341,19 @@
       </c>
       <c r="E403" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" s="3" t="inlineStr">
         <is>
-          <t>212200</t>
+          <t>212133</t>
         </is>
       </c>
       <c r="B404" s="3" t="inlineStr">
         <is>
-          <t>Athian Madut Athian Dut</t>
+          <t>Mohammed Kashif Saleem</t>
         </is>
       </c>
       <c r="C404" s="3" t="inlineStr">
@@ -11368,19 +11368,19 @@
       </c>
       <c r="E404" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" s="4" t="inlineStr">
         <is>
-          <t>212209</t>
+          <t>212200</t>
         </is>
       </c>
       <c r="B405" s="4" t="inlineStr">
         <is>
-          <t>لازرى باسكاندا</t>
+          <t>Athian Madut Athian Dut</t>
         </is>
       </c>
       <c r="C405" s="4" t="inlineStr">
@@ -11395,19 +11395,19 @@
       </c>
       <c r="E405" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" s="3" t="inlineStr">
         <is>
-          <t>212218</t>
+          <t>212209</t>
         </is>
       </c>
       <c r="B406" s="3" t="inlineStr">
         <is>
-          <t>Abdul Arham</t>
+          <t>لازرى باسكاندا</t>
         </is>
       </c>
       <c r="C406" s="3" t="inlineStr">
@@ -11422,19 +11422,19 @@
       </c>
       <c r="E406" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" s="4" t="inlineStr">
         <is>
-          <t>212231</t>
+          <t>212218</t>
         </is>
       </c>
       <c r="B407" s="4" t="inlineStr">
         <is>
-          <t>Fathima Sana Ansari</t>
+          <t>Abdul Arham</t>
         </is>
       </c>
       <c r="C407" s="4" t="inlineStr">
@@ -11449,19 +11449,19 @@
       </c>
       <c r="E407" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" s="3" t="inlineStr">
         <is>
-          <t>212238</t>
+          <t>212231</t>
         </is>
       </c>
       <c r="B408" s="3" t="inlineStr">
         <is>
-          <t>Arifuddeen Idris Ibrahim</t>
+          <t>Fathima Sana Ansari</t>
         </is>
       </c>
       <c r="C408" s="3" t="inlineStr">
@@ -11476,19 +11476,19 @@
       </c>
       <c r="E408" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" s="4" t="inlineStr">
         <is>
-          <t>212247</t>
+          <t>212238</t>
         </is>
       </c>
       <c r="B409" s="4" t="inlineStr">
         <is>
-          <t>Aastha Attri</t>
+          <t>Arifuddeen Idris Ibrahim</t>
         </is>
       </c>
       <c r="C409" s="4" t="inlineStr">
@@ -11503,19 +11503,19 @@
       </c>
       <c r="E409" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" s="3" t="inlineStr">
         <is>
-          <t>212316</t>
+          <t>212247</t>
         </is>
       </c>
       <c r="B410" s="3" t="inlineStr">
         <is>
-          <t>William Marial Mayek Bol</t>
+          <t>Aastha Attri</t>
         </is>
       </c>
       <c r="C410" s="3" t="inlineStr">
@@ -11530,19 +11530,19 @@
       </c>
       <c r="E410" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" s="4" t="inlineStr">
         <is>
-          <t>212392</t>
+          <t>212316</t>
         </is>
       </c>
       <c r="B411" s="4" t="inlineStr">
         <is>
-          <t>Joseph Malual Mareng Ajou</t>
+          <t>William Marial Mayek Bol</t>
         </is>
       </c>
       <c r="C411" s="4" t="inlineStr">
@@ -11557,19 +11557,19 @@
       </c>
       <c r="E411" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" s="3" t="inlineStr">
         <is>
-          <t>212434</t>
+          <t>212392</t>
         </is>
       </c>
       <c r="B412" s="3" t="inlineStr">
         <is>
-          <t>Athou Philp Marial Yuot</t>
+          <t>Joseph Malual Mareng Ajou</t>
         </is>
       </c>
       <c r="C412" s="3" t="inlineStr">
@@ -11584,19 +11584,19 @@
       </c>
       <c r="E412" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" s="4" t="inlineStr">
         <is>
-          <t>220852</t>
+          <t>212434</t>
         </is>
       </c>
       <c r="B413" s="4" t="inlineStr">
         <is>
-          <t>سلامة محمد</t>
+          <t>Athou Philp Marial Yuot</t>
         </is>
       </c>
       <c r="C413" s="4" t="inlineStr">
@@ -11611,19 +11611,19 @@
       </c>
       <c r="E413" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" s="3" t="inlineStr">
         <is>
-          <t>221563</t>
+          <t>220852</t>
         </is>
       </c>
       <c r="B414" s="3" t="inlineStr">
         <is>
-          <t>زينب انيس حيدرى</t>
+          <t>سلامة محمد</t>
         </is>
       </c>
       <c r="C414" s="3" t="inlineStr">
@@ -11638,19 +11638,19 @@
       </c>
       <c r="E414" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="A415" s="4" t="inlineStr">
         <is>
-          <t>221669</t>
+          <t>221563</t>
         </is>
       </c>
       <c r="B415" s="4" t="inlineStr">
         <is>
-          <t>فرحان يوسف شيخ</t>
+          <t>زينب انيس حيدرى</t>
         </is>
       </c>
       <c r="C415" s="4" t="inlineStr">
@@ -11665,19 +11665,19 @@
       </c>
       <c r="E415" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="A416" s="3" t="inlineStr">
         <is>
-          <t>221738</t>
+          <t>221669</t>
         </is>
       </c>
       <c r="B416" s="3" t="inlineStr">
         <is>
-          <t>شعيب يوسف</t>
+          <t>فرحان يوسف شيخ</t>
         </is>
       </c>
       <c r="C416" s="3" t="inlineStr">
@@ -11692,19 +11692,19 @@
       </c>
       <c r="E416" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" s="4" t="inlineStr">
         <is>
-          <t>221750</t>
+          <t>221738</t>
         </is>
       </c>
       <c r="B417" s="4" t="inlineStr">
         <is>
-          <t>احمد كاملي مير</t>
+          <t>شعيب يوسف</t>
         </is>
       </c>
       <c r="C417" s="4" t="inlineStr">
@@ -11719,19 +11719,19 @@
       </c>
       <c r="E417" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" s="3" t="inlineStr">
         <is>
-          <t>221825</t>
+          <t>221750</t>
         </is>
       </c>
       <c r="B418" s="3" t="inlineStr">
         <is>
-          <t>جويرية فوديو موسى</t>
+          <t>احمد كاملي مير</t>
         </is>
       </c>
       <c r="C418" s="3" t="inlineStr">
@@ -11746,19 +11746,19 @@
       </c>
       <c r="E418" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" s="4" t="inlineStr">
         <is>
-          <t>221867</t>
+          <t>221825</t>
         </is>
       </c>
       <c r="B419" s="4" t="inlineStr">
         <is>
-          <t>حماد احمد خان</t>
+          <t>جويرية فوديو موسى</t>
         </is>
       </c>
       <c r="C419" s="4" t="inlineStr">
@@ -11773,19 +11773,19 @@
       </c>
       <c r="E419" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" s="3" t="inlineStr">
         <is>
-          <t>221892</t>
+          <t>221867</t>
         </is>
       </c>
       <c r="B420" s="3" t="inlineStr">
         <is>
-          <t>عائشة على حمزة</t>
+          <t>حماد احمد خان</t>
         </is>
       </c>
       <c r="C420" s="3" t="inlineStr">
@@ -11800,19 +11800,19 @@
       </c>
       <c r="E420" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" s="4" t="inlineStr">
         <is>
-          <t>221893</t>
+          <t>221892</t>
         </is>
       </c>
       <c r="B421" s="4" t="inlineStr">
         <is>
-          <t>هولى امانويل لوكيرى كمورة</t>
+          <t>عائشة على حمزة</t>
         </is>
       </c>
       <c r="C421" s="4" t="inlineStr">
@@ -11827,19 +11827,19 @@
       </c>
       <c r="E421" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" s="3" t="inlineStr">
         <is>
-          <t>221907</t>
+          <t>221893</t>
         </is>
       </c>
       <c r="B422" s="3" t="inlineStr">
         <is>
-          <t>اطهر بشير مير</t>
+          <t>هولى امانويل لوكيرى كمورة</t>
         </is>
       </c>
       <c r="C422" s="3" t="inlineStr">
@@ -11854,19 +11854,19 @@
       </c>
       <c r="E422" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" s="4" t="inlineStr">
         <is>
-          <t>221921</t>
+          <t>221907</t>
         </is>
       </c>
       <c r="B423" s="4" t="inlineStr">
         <is>
-          <t>مديحة نزير</t>
+          <t>اطهر بشير مير</t>
         </is>
       </c>
       <c r="C423" s="4" t="inlineStr">
@@ -11881,19 +11881,19 @@
       </c>
       <c r="E423" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" s="3" t="inlineStr">
         <is>
-          <t>221943</t>
+          <t>221921</t>
         </is>
       </c>
       <c r="B424" s="3" t="inlineStr">
         <is>
-          <t>جيمس افانديت مجوك هانشيانق</t>
+          <t>مديحة نزير</t>
         </is>
       </c>
       <c r="C424" s="3" t="inlineStr">
@@ -11908,19 +11908,19 @@
       </c>
       <c r="E424" s="3" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" s="4" t="inlineStr">
         <is>
-          <t>221975</t>
+          <t>221943</t>
         </is>
       </c>
       <c r="B425" s="4" t="inlineStr">
         <is>
-          <t>ازاكو طونقكوك كوكلونق ماكير</t>
+          <t>جيمس افانديت مجوك هانشيانق</t>
         </is>
       </c>
       <c r="C425" s="4" t="inlineStr">
@@ -11935,34 +11935,61 @@
       </c>
       <c r="E425" s="4" t="inlineStr">
         <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="A426" s="3" t="inlineStr">
         <is>
+          <t>221975</t>
+        </is>
+      </c>
+      <c r="B426" s="3" t="inlineStr">
+        <is>
+          <t>ازاكو طونقكوك كوكلونق ماكير</t>
+        </is>
+      </c>
+      <c r="C426" s="3" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="D426" s="3" t="inlineStr">
+        <is>
+          <t>A1-F2</t>
+        </is>
+      </c>
+      <c r="E426" s="3" t="inlineStr">
+        <is>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" s="4" t="inlineStr">
+        <is>
           <t>221976</t>
         </is>
       </c>
-      <c r="B426" s="3" t="inlineStr">
+      <c r="B427" s="4" t="inlineStr">
         <is>
           <t>مابور مايور شوال ميان</t>
         </is>
       </c>
-      <c r="C426" s="3" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="D426" s="3" t="inlineStr">
+      <c r="C427" s="4" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="D427" s="4" t="inlineStr">
         <is>
           <t>A1-F2</t>
         </is>
       </c>
-      <c r="E426" s="3" t="inlineStr">
-        <is>
-          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102513.xlsx</t>
+      <c r="E427" s="4" t="inlineStr">
+        <is>
+          <t>Y4_B2526_General_&amp;_Special_Surgery_1_A1_reference_data_D01062026T102618.xlsx</t>
         </is>
       </c>
     </row>

</xml_diff>